<commit_message>
Added New and Left employee logic
Added New and Left employee logic
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PYTHON WORKING\attendence_working\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nazeer Ahmed Khan\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B937906F-9A0C-47C8-8125-A2B85731D3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC9EF9A-4BDD-4D29-A161-6E048C1C3DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{86A33D8E-3FC0-4676-BB1D-2A735C88F353}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$56</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="91">
   <si>
     <t>CODE</t>
   </si>
@@ -288,7 +291,16 @@
     <t>Kamran</t>
   </si>
   <si>
-    <t>TOTAL DAYS September 2025</t>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>NEW</t>
+  </si>
+  <si>
+    <t>TOTAL DAYS</t>
+  </si>
+  <si>
+    <t>Date</t>
   </si>
 </sst>
 </file>
@@ -299,7 +311,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
       <color theme="1"/>
@@ -334,6 +346,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -384,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -409,6 +427,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -724,16 +745,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189B965E-FE38-487F-86A9-CB28C9D4D4A6}">
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="3.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.35546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="39" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="31" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -747,7 +769,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>50</v>
@@ -761,8 +783,14 @@
       <c r="I1" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -790,8 +818,10 @@
       <c r="I2" s="9">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J2" s="10"/>
+      <c r="K2" s="11"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -817,8 +847,10 @@
       <c r="I3" s="6">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J3" s="6"/>
+      <c r="K3" s="11"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -844,8 +876,10 @@
       <c r="I4" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J4" s="6"/>
+      <c r="K4" s="11"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -873,8 +907,10 @@
       <c r="I5" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J5" s="6"/>
+      <c r="K5" s="11"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -902,8 +938,10 @@
       <c r="I6" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J6" s="6"/>
+      <c r="K6" s="11"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -916,9 +954,7 @@
       <c r="D7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="6">
-        <v>30</v>
-      </c>
+      <c r="E7" s="9"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6">
         <v>1</v>
@@ -929,8 +965,14 @@
       <c r="I7" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J7" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K7" s="12">
+        <v>45971</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -943,9 +985,7 @@
       <c r="D8" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="6">
-        <v>30</v>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6">
         <v>1</v>
@@ -956,8 +996,14 @@
       <c r="I8" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J8" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K8" s="12">
+        <v>45976</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -985,8 +1031,10 @@
       <c r="I9" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J9" s="6"/>
+      <c r="K9" s="11"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1012,8 +1060,10 @@
       <c r="I10" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J10" s="6"/>
+      <c r="K10" s="11"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1041,8 +1091,10 @@
       <c r="I11" s="6">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J11" s="6"/>
+      <c r="K11" s="11"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1068,8 +1120,10 @@
       <c r="I12" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J12" s="6"/>
+      <c r="K12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1095,8 +1149,10 @@
       <c r="I13" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J13" s="6"/>
+      <c r="K13" s="11"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1122,8 +1178,10 @@
       <c r="I14" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J14" s="6"/>
+      <c r="K14" s="11"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1149,8 +1207,10 @@
       <c r="I15" s="6">
         <v>31</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J15" s="6"/>
+      <c r="K15" s="11"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1178,8 +1238,10 @@
       <c r="I16" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J16" s="6"/>
+      <c r="K16" s="11"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1205,8 +1267,10 @@
       <c r="I17" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J17" s="6"/>
+      <c r="K17" s="11"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1232,8 +1296,10 @@
       <c r="I18" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J18" s="6"/>
+      <c r="K18" s="11"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1259,8 +1325,10 @@
       <c r="I19" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J19" s="6"/>
+      <c r="K19" s="11"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1288,8 +1356,10 @@
       <c r="I20" s="6">
         <v>31</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J20" s="6"/>
+      <c r="K20" s="11"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1315,8 +1385,10 @@
       <c r="I21" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J21" s="6"/>
+      <c r="K21" s="11"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1342,8 +1414,10 @@
       <c r="I22" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J22" s="6"/>
+      <c r="K22" s="11"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1369,8 +1443,10 @@
       <c r="I23" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J23" s="6"/>
+      <c r="K23" s="11"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1396,8 +1472,10 @@
       <c r="I24" s="6">
         <v>32</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J24" s="6"/>
+      <c r="K24" s="11"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1425,8 +1503,10 @@
       <c r="I25" s="6">
         <v>31</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J25" s="6"/>
+      <c r="K25" s="11"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1454,8 +1534,10 @@
       <c r="I26" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J26" s="6"/>
+      <c r="K26" s="11"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1481,8 +1563,10 @@
       <c r="I27" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J27" s="6"/>
+      <c r="K27" s="11"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -1508,8 +1592,10 @@
       <c r="I28" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J28" s="6"/>
+      <c r="K28" s="11"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1535,8 +1621,10 @@
       <c r="I29" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J29" s="6"/>
+      <c r="K29" s="11"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -1564,8 +1652,10 @@
       <c r="I30" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J30" s="6"/>
+      <c r="K30" s="11"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -1591,8 +1681,10 @@
       <c r="I31" s="6">
         <v>32</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J31" s="6"/>
+      <c r="K31" s="11"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -1618,8 +1710,10 @@
       <c r="I32" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J32" s="6"/>
+      <c r="K32" s="11"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -1645,8 +1739,10 @@
       <c r="I33" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J33" s="6"/>
+      <c r="K33" s="11"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1674,8 +1770,10 @@
       <c r="I34" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J34" s="6"/>
+      <c r="K34" s="11"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -1701,8 +1799,10 @@
       <c r="I35" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J35" s="6"/>
+      <c r="K35" s="11"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -1728,8 +1828,10 @@
       <c r="I36" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J36" s="6"/>
+      <c r="K36" s="11"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -1755,8 +1857,10 @@
       <c r="I37" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J37" s="6"/>
+      <c r="K37" s="11"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -1782,8 +1886,10 @@
       <c r="I38" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J38" s="6"/>
+      <c r="K38" s="11"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -1811,8 +1917,10 @@
       <c r="I39" s="6">
         <v>31</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J39" s="6"/>
+      <c r="K39" s="11"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -1838,8 +1946,10 @@
       <c r="I40" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J40" s="6"/>
+      <c r="K40" s="11"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -1867,8 +1977,10 @@
       <c r="I41" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J41" s="6"/>
+      <c r="K41" s="11"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -1894,8 +2006,10 @@
       <c r="I42" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J42" s="6"/>
+      <c r="K42" s="11"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -1921,8 +2035,10 @@
       <c r="I43" s="6">
         <v>32</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J43" s="6"/>
+      <c r="K43" s="11"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -1948,8 +2064,10 @@
       <c r="I44" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J44" s="6"/>
+      <c r="K44" s="11"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -1977,8 +2095,10 @@
       <c r="I45" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J45" s="6"/>
+      <c r="K45" s="11"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -2004,8 +2124,10 @@
       <c r="I46" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J46" s="6"/>
+      <c r="K46" s="11"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -2031,8 +2153,10 @@
       <c r="I47" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J47" s="6"/>
+      <c r="K47" s="11"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -2045,9 +2169,7 @@
       <c r="D48" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E48" s="6">
-        <v>30</v>
-      </c>
+      <c r="E48" s="6"/>
       <c r="F48" s="6"/>
       <c r="G48" s="6">
         <v>1</v>
@@ -2058,8 +2180,14 @@
       <c r="I48" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J48" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K48" s="12">
+        <v>45981</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -2087,8 +2215,10 @@
       <c r="I49" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J49" s="6"/>
+      <c r="K49" s="11"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -2114,8 +2244,10 @@
       <c r="I50" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J50" s="6"/>
+      <c r="K50" s="11"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -2143,8 +2275,10 @@
       <c r="I51" s="6">
         <v>29</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J51" s="6"/>
+      <c r="K51" s="11"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -2170,8 +2304,10 @@
       <c r="I52" s="6">
         <v>32</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J52" s="6"/>
+      <c r="K52" s="11"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -2197,8 +2333,10 @@
       <c r="I53" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J53" s="6"/>
+      <c r="K53" s="11"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -2211,9 +2349,7 @@
       <c r="D54" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E54" s="6">
-        <v>30</v>
-      </c>
+      <c r="E54" s="6"/>
       <c r="F54" s="6"/>
       <c r="G54" s="6">
         <v>1</v>
@@ -2224,8 +2360,14 @@
       <c r="I54" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J54" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K54" s="12">
+        <v>45682</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -2253,8 +2395,10 @@
       <c r="I55" s="6">
         <v>27</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J55" s="6"/>
+      <c r="K55" s="11"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -2280,8 +2424,11 @@
       <c r="I56" s="6">
         <v>29</v>
       </c>
+      <c r="J56" s="6"/>
+      <c r="K56" s="11"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K56" xr:uid="{189B965E-FE38-487F-86A9-CB28C9D4D4A6}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>